<commit_message>
added main.py to run all the state
</commit_message>
<xml_diff>
--- a/src/scrapers/output_scrape/combined/requirements_all_states.xlsx
+++ b/src/scrapers/output_scrape/combined/requirements_all_states.xlsx
@@ -2856,165 +2856,70 @@
 Under the SkillSelect model, the Department of Home Affairs invite skilled workers to apply for a Skilled Nominated visa (subclass 190) based on the claims presented in their expression of interest (EOI) in SkillSelect.
 The applicant must satisfy most criteria specified in the points test at the time of invitation.
 AGE
-[Age]
-[Points]
-  at least 18 but less than 25 years
-  25
-  at least  25 but less than 33 years
-  30
-  at least  33 but less than 40 years
-  25
-  at least  40 but less than 45 years
-  15
+[Age] = at least 18 but less than 25 years   [Points] = 25
+[Age] = at least  25 but less than 33 years   [Points] = 30
+[Age] = at least  33 but less than 40 years   [Points] = 25
+[Age] = at least  40 but less than 45 years   [Points] = 15
 ENGLISH LANGUAGE SKILLS
-[English]
-[Points]
-  Competent English
-  0
-  Proficient English
-  10
-  Superior English
-  20
+[English] = Competent English   [Points] = 0
+[English] = Proficient English   [Points] = 10
+[English] = Superior English   [Points] = 20
 English language skills
 SKILLED EMPLOYMENT EXPERIENCE
 OVERSEAS SKILLED EMPLOYMENT – (OUTSIDE AUSTRALIA)
-[Number of years]
-[Points]
-  Less than 3 years
-  0
-  At least 3 but less than 5 years
-  5
-  At least 5 but less than 8 years
-  10
-  At least 8 years
-  15
+[Number of years] = Less than 3 years   [Points] = 0
+[Number of years] = At least 3 but less than 5 years   [Points] = 5
+[Number of years] = At least 5 but less than 8 years   [Points] = 10
+[Number of years] = At least 8 years   [Points] = 15
 AUSTRALIAN SKILLED EMPLOYMENT – (IN AUSTRALIA)
-[Number of years]
-[Points]
-  Less than 1 year
-  0
-  At least 1 but less than 3 years
-  5
-  At least 3 but less than 5 years
-  10
-  At least 5 but less than 8 years
-  15
-  At least 8 years
-  20
-• You can only claim points for employment if the employment was in your nominated skilled occupation or a closely related skilled occupation; and you were employed for the relevant periods set out in the table, in the 10 years before you are invited to apply.
-• For any Australian employment you must have held asubstantive visaor aBridging AorBridging Bvisa and complied with the conditions of that visa to be eligible for points.
+[Number of years] = Less than 1 year   [Points] = 0
+[Number of years] = At least 1 but less than 3 years   [Points] = 5
+[Number of years] = At least 3 but less than 5 years   [Points] = 10
+[Number of years] = At least 5 but less than 8 years   [Points] = 15
+[Number of years] = At least 8 years   [Points] = 20
 Employed means engaged in an occupation for remuneration for at least 20 hours a week.
 Closely-related occupations must be:
-• in the same ANZSCO Unit Group or
-• consistent with a career advancement pathway or
-• recognised by an assessing authority that it is closely related to your nominated occupation, as part of your skills assessment
 Under the points test there is a cap on the number of points that can be awarded for employment experience. The maximum number of points that can be awarded is 20, this means that even if you score more than 20 combined points for your employment experience only 20 points will be awarded.
 EDUCATIONAL QUALIFICATIONS
-[Requirement]
-[Points]
-  A Doctorate from an Australian educational institution or a Doctorate from another educational institution, that is of arecognised standard.
-  20
-  At least a Bachelor degree from an Australian educational institution or at least a Bachelor qualification, from another educational institution, that is of arecognised standard.
-  15
-  A diploma or trade qualification from an Australian educational institution.
-  10
-  Attained a qualification or award recognised by the relevant assessing authority for your nominated skilled occupation as being suitable for that occupation
-  10
+[Requirement] = A Doctorate from an Australian educational institution or a Doctorate from another educational institution, that is of a recognised standard .   [Points] = 20
+[Requirement] = At least a Bachelor degree from an Australian educational institution or at least a Bachelor qualification, from another educational institution, that is of a recognised standard .   [Points] = 15
+[Requirement] = A diploma or trade qualification from an Australian educational institution.   [Points] = 10
+[Requirement] = Attained a qualification or award recognised by the relevant assessing authority for your nominated skilled occupation as being suitable for that occupation   [Points] = 10
 For points based migration you will receive points for your highest qualification only.
 RECOGNITION OF YOUR QUALIFICATIONS
-The authority undertaking your skills assessment may determine if your qualifications are comparable to the relevant Australian qualification. Assessing authorities are listed against your occupation in the relevant list ofeligible skilled occupations. You must have obtained this recognition at the time you are invited to apply for a visa.
+The authority undertaking your skills assessment may determine if your qualifications are comparable to the relevant Australian qualification. Assessing authorities are listed against your occupation in the relevant list of eligible skilled occupations . You must have obtained this recognition at the time you are invited to apply for a visa.
 If you hold an overseas qualification at bachelor level or above and your skills assessing authority did not offer an opinion on that qualification then it is open to you to contact Vocational Education Training and Assessment Services (VETASSESS) for advice.
 VETASSESS can provide an assessment of the comparative educational level of these qualifications against the Australian Qualifications Framework (AQF). Advice from VETASSESS should be provided with your application to support your claim for these points.
-To obtain an assessment  contactVocational Education Training and Assessment Services.
+To obtain an assessment  contact Vocational Education Training and Assessment Services .
 DOCTORAL REQUIREMENTS (PHD)
 You can only be awarded points for a doctoral degree if you have completed a qualification at the relevant level, that is,  a Doctor of Philosophy (PhD). You cannot claim these points for the award of other qualifications that give you the right to use to the title of Doctor (that is, general practitioner, dentist, vet).
 SPECIALIST EDUCATION QUALIFICATION
-[Requirement]
-[Points]
-  A Masters degree by research or a Doctorate degree from an Australian educational institution that included at least 2academic years studyin a relevant field.
-  10
+[Requirement] = A Masters degree by research or a Doctorate degree from an Australian educational institution that included at least 2 academic years study in a relevant field.   [Points] = 10
 The postgraduate degree by research (doctorate or masters) must be awarded from an Australian education institution after at least two academic years of study in the following science, technology, engineering, mathematics or specified information and communication technology (ICT) fields:
 Natural and physical sciences
-• biological sciences
-• chemical sciences
-• earth sciences
-• mathematical sciences
-• natural and physical sciences
-• other natural and physical sciences
-• physics and astronomy
 Information technology
-• computer science
-• information systems
-• information technology
-• other information technology
 Engineering and related technologies
-• aerospace engineering and technology
-• civil engineering
-• electrical and electronic engineering and technology
-• engineering and related technologies
-• geomatics engineering
-• manufacturing engineering and technology
-• maritime engineering and technology
-• mechanical and industrial engineering and technology
-• other engineering and related technologies
-• process and resources engineering.
-To determine whether your qualification is eligible, see theCRICOSwebsite.
+To determine whether your qualification is eligible, see the CRICOS website.
 AUSTRALIAN STUDY REQUIREMENT
-[Requirement]
-[Points]
-  Meet the Australian study requirement
-  5
-You must have at least 1 degree, diploma or trade qualification from an Australian educational institution that meets theAustralian study requirement.
+[Requirement] = Meet the Australian study requirement   [Points] = 5
+You must have at least 1 degree, diploma or trade qualification from an Australian educational institution that meets the Australian study requirement.
 PROFESSIONAL YEAR IN AUSTRALIA
-[Requirement]
-[Points]
-  Completion of a Professional Year in Australia
-  5
+[Requirement] = Completion of a Professional Year in Australia   [Points] = 5
 At the time of invitation to apply, you had completed a Professional Year. To be eligible for the award of these points your Professional Year must have been in Accounting, ICT/Computing or Engineering, and:
-• in your nominated occupation or a closely related occupation
-• completed over a period of at least 12 months
-• completed in Australia in the four years before you are invited to apply for a visa*
-• provided by one of these organisations:theAustralian Computer SocietyCPA AustraliaChartered Accountants Australia and New ZealandtheInstitute of Public Accountants(formerly the National Institute of Accountants)Engineers Australia.
-• theAustralian Computer Society
-• CPA Australia
-• Chartered Accountants Australia and New Zealand
-• theInstitute of Public Accountants(formerly the National Institute of Accountants)
-• Engineers Australia.
 * Where a Professional Year program was completed, meaning finished, within the 48 month period prior to the time of invitation, you may be awarded 5 points. To avoid any doubt, you could have commenced the Professional Year at a time before the 48 months prior to invitation. The time you “completed” a Professional Year is the date listed on your official Record of Completion which is issued by the authorised body or Professional Year program delivery partner.
 CREDENTIALLED COMMUNITY LANGUAGE
-[Requirement]
-[Points]
-  Hold a recognised qualification in a credentialled community language
-  5
-To be credentialled in a community language and eligible for the award of points you must have been accredited at the paraprofessional level or above, certified at the certified provisional level or above, or have a community language credential for interpreting or translating by theNational Accreditation Authority for Translators and Interpreters.
+[Requirement] = Hold a recognised qualification in a credentialled community language   [Points] = 5
+To be credentialled in a community language and eligible for the award of points you must have been accredited at the paraprofessional level or above, certified at the certified provisional level or above, or have a community language credential for interpreting or translating by the National Accreditation Authority for Translators and Interpreters .
 STUDY IN REGIONAL AUSTRALIA
-[Requirement]
-[Points]
-  You must have at least 1 degree, diploma or trade qualification from an Australian educational institution that satisfies theAustralian study requirementobtained while living and studying in an eligible area of regional Australia
-  5
+[Requirement] = You must have at least 1 degree, diploma or trade qualification from an Australian educational institution that satisfies the Australian study requirement obtained while living and studying in an eligible area of regional Australia   [Points] = 5
 To be eligible for the award of points your educational qualification:
-• must meet theAustralian study requirement
-• have been obtained while you lived in, and studied at a campus in a designated regional area
-• not include study undertaken by distance education
 PARTNER SKILLS
-[Requirement]
-[Points]
-  Yourspouseorde factopartner must also be an applicant for this visa and meet age, English and skill criteriaFor you to be eligible for the award of these points yourpartnermust be an applicant for the same visa subclass and must not be an Australian permanent resident or an Australian citizen.  Additionally, you will need to provide evidence that when you were invited to apply for this visa that they:were under 45 years oldhadcompetent Englishhad nominated a skilled occupation that is on the same skilled occupation list as your nominated skilled occupationhad a suitable skills assessment from the relevant assessing authority for their nominated skilled occupation, and the assessment wasn’t for a Subclass 485 visa.
-• were under 45 years old
-• hadcompetent English
-• had nominated a skilled occupation that is on the same skilled occupation list as your nominated skilled occupation
-• had a suitable skills assessment from the relevant assessing authority for their nominated skilled occupation, and the assessment wasn’t for a Subclass 485 visa.
-  10
-  Your spouse or de facto partner must also be an applicant for this visa and hascompetent EnglishFor you to be eligible for the award of these points your partner must be an applicant for the same visa subclass and must not be an Australian permanent resident or an Australian citizen.
-  5
-  You are single or your partner is an Australian citizen or permanent resident*
-  10
+[Requirement] = Your spouse or de facto partner must also be an applicant for this visa and meet age, English and skill criteria For you to be eligible for the award of these points your partner must be an applicant for the same visa subclass and must not be an Australian permanent resident or an Australian citizen.  Additionally, you will need to provide evidence that when you were invited to apply for this visa that they: were under 45 years old had competent English had nominated a skilled occupation that is on the same skilled occupation list as your nominated skilled occupation had a suitable skills assessment from the relevant assessing authority for their nominated skilled occupation, and the assessment wasn’t for a Subclass 485 visa.   [Points] = 10
+[Requirement] = Your spouse or de facto partner must also be an applicant for this visa and has competent English For you to be eligible for the award of these points your partner must be an applicant for the same visa subclass and must not be an Australian permanent resident or an Australian citizen.   [Points] = 5
+[Requirement] = You are single or your partner is an Australian citizen or permanent resident*   [Points] = 10
 *If your marital status changes during the processing of your visa, we may not award you points for this item. We do not assess this item as at the time of invitation.
 NOMINATION
-[Requirement]
-[Points]
-  You were invited to apply for a Subclass 190 (Skilled — Nominated) visa and the nominating State or Territory government agency has not withdrawn the nomination
-  5
+[Requirement] = You were invited to apply for a Subclass 190 (Skilled — Nominated) visa and the nominating State or Territory government agency has not withdrawn the nomination   [Points] = 5
 You must be nominated to be invited to apply for this visa. Provided your nomination remains in effect, you may be eligible for the award of these points.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
added function to combine all the excel state to excel file
</commit_message>
<xml_diff>
--- a/src/scrapers/output_scrape/combined/requirements_all_states.xlsx
+++ b/src/scrapers/output_scrape/combined/requirements_all_states.xlsx
@@ -7,7 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACT" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NT" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NSW" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QLD" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SA" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIC" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WA" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +32,23 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +63,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -416,23 +436,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
     <col width="80" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="80" customWidth="1" min="7" max="7"/>
-    <col width="80" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="40" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -466,59 +478,19 @@
           <t>service fee</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>requirements</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Detail Requirements</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>state_code</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>state_stream</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>tse</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>tsg</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>ter</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>tbo</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="409" customHeight="1">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ACT</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>190</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>The Skilled Nominated Visa (subclass 190) lets you live and work in Australia as a permanent resident. You must be nominated by a State or Territory government. Nomination triggers the visa invitation from the Department of Home Affairs.
 Two year commitment - If you are nominated by the ACT to apply for a 190 visa, you must live and work in Canberra for at least two years from visa grant, or if you are moving from overseas, date of arrival in Canberra.
@@ -534,7 +506,7 @@
 Overseas applicant eligibility</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Department of Home Affairs Criteria: you meet the relevant Department of Home Affairs Criteria and can apply for your visa. You must meet this criterion when you submit your Canberra Matrix and continue to do so until you receive ACT nomination. This includes having a valid English test and Skill Assessment.
 • Your English test and Skill Assessment must be valid at date of Canberra Matrix submission and at date of ACT nomination.
@@ -556,7 +528,7 @@
 Service fee : $300</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Department of Home Affairs Criteria: you meet the relevant Department of Home Affairs Criteria and can apply for your visa. You must meet this criterion when you submit your Canberra Matrix and continue to do so until you receive ACT nomination. This includes having a valid English test and Skill Assessment.
 • Your English test and Skill Assessment must be valid at date of Canberra Matrix submission and at date of ACT nomination.
@@ -582,32 +554,24 @@
 Service Fee : $300 Your supporting documentation must evidence your eligibility to apply for ACT nomination and any Matrix score claimed. Please refer to the key document checklist for more information on what documents you need to include.</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>$300 (overseas), $300 (canberra)</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr"/>
-      <c r="H2" s="1" t="inlineStr"/>
-      <c r="I2" s="1" t="inlineStr"/>
-      <c r="J2" s="1" t="inlineStr"/>
-      <c r="K2" s="1" t="inlineStr"/>
-      <c r="L2" s="1" t="inlineStr"/>
-      <c r="M2" s="1" t="inlineStr"/>
-      <c r="N2" s="1" t="inlineStr"/>
     </row>
     <row r="3" ht="409" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>ACT</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>491</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>The Skilled Regional Work Visa (subclass 491) is a five year provisional visa for skilled workers to live and work in regional Australia. You must be nominated by a state or territory government. Nomination triggers the visa invitation from the Department of Home Affairs.
 Two year commitment - If you are nominated by the ACT to apply for a 491 visa, you must live and work in Canberra for at least two years from visa grant, or if you are moving from overseas, date of arrival in Canberra.
@@ -623,7 +587,7 @@
 Overseas applicant eligibility</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Department of Home Affairs Criteria: you meet the relevant Department of Home Affairs Criteria and can apply for your visa. You must meet this criterion when you submit your Canberra Matrix and continue to do so until you receive ACT nomination. This includes having a valid English test and Skill Assessment.
 • Your English test and Skill Assessment must be valid at date of Canberra Matrix submission and at date of ACT nomination.
@@ -643,7 +607,7 @@
 Service fee : $300</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Department of Home Affairs Criteria: you meet the relevant Department of Home Affairs Criteria and can apply for your visa. You must meet this criterion when you submit your Canberra Matrix and continue to do so until you receive ACT nomination. This includes having a valid English test and Skill Assessment.
 • Your English test and Skill Assessment must be valid at date of Canberra Matrix submission and at date of ACT nomination.
@@ -668,40 +632,66 @@
 Service Fee : $300</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>$300 (overseas), $300 (canberra)</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr"/>
-      <c r="H3" s="1" t="inlineStr"/>
-      <c r="I3" s="1" t="inlineStr"/>
-      <c r="J3" s="1" t="inlineStr"/>
-      <c r="K3" s="1" t="inlineStr"/>
-      <c r="L3" s="1" t="inlineStr"/>
-      <c r="M3" s="1" t="inlineStr"/>
-      <c r="N3" s="1" t="inlineStr"/>
     </row>
-    <row r="4" ht="409" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>state code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>state stream</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>requirements</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>service fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="409" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>NT</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Northern_Territory</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr"/>
-      <c r="D4" s="1" t="inlineStr"/>
-      <c r="E4" s="1" t="inlineStr"/>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>WHAT IS A NORTHERN TERRITORY GOVERNMENT NOMINATION?
 Australia's Northern Territory (NT) Government participates in the Skilled Work Regional (Provisional) (subclass 491) visa and Skilled Nominated (subclass 190) visa schemes.
@@ -736,60 +726,90 @@
 The NT Government does not approve or grant visas.</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr"/>
-      <c r="I4" s="1" t="inlineStr"/>
-      <c r="J4" s="1" t="inlineStr"/>
-      <c r="K4" s="1" t="inlineStr"/>
-      <c r="L4" s="1" t="inlineStr"/>
-      <c r="M4" s="1" t="inlineStr"/>
-      <c r="N4" s="1" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="5" ht="45" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>NT</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Northern_Territory_Offshore</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr"/>
-      <c r="D5" s="1" t="inlineStr"/>
-      <c r="E5" s="1" t="inlineStr"/>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G5" s="1" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>This list is only applicable for those applying for Northern Territory (NT) nomination from outside Australia, under the priority occupation stream . If you are currently living in the NT or living overseas and applying under the NT family stream or the NT job offer stream, you can nominate any occupation on the national eligibility list for the subclass 491 visa on the Australian Government Department of Home Affairs website .
 The Department of Home Affairs utilise the 2013 ANZSCO version for occupation descriptions for the skilled visa subclasses 491 and 190.
 Please note: Offshore applicants will generally only be considered for a nomination for a subclass 491 visa.</t>
         </is>
       </c>
-      <c r="H5" s="1" t="inlineStr"/>
-      <c r="I5" s="1" t="inlineStr"/>
-      <c r="J5" s="1" t="inlineStr"/>
-      <c r="K5" s="1" t="inlineStr"/>
-      <c r="L5" s="1" t="inlineStr"/>
-      <c r="M5" s="1" t="inlineStr"/>
-      <c r="N5" s="1" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="6" ht="255" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>state code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>state stream</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>General Requirements</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Detail Requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="255" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>190</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Visa eligibility - Ensure you meet all visa requirements outlined by Home Affairs for this visa.
 Skills assessment - Have a valid skills assessment for an occupation that is both:
@@ -801,11 +821,7 @@
 • Residing offshore and have continuously resided offshore for a minimum period of six months.</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr"/>
-      <c r="E6" s="1" t="inlineStr"/>
-      <c r="F6" s="1" t="inlineStr"/>
-      <c r="G6" s="1" t="inlineStr"/>
-      <c r="H6" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Check Eligibility : Before submitting your EOI in SkillSelect, ensure you meet both the visa and NSW nomination eligibility requirements.
 Submit Your EOI : If you meet the criteria, submit an EOI in SkillSelect. Should you be invited to apply, you need to support every claim in your EOI with valid (i.e. non-expired) documents.
@@ -818,36 +834,26 @@
 Submission Date : The date you submit or amend your SkillSelect EOI does not affect your likelihood of being invited.</t>
         </is>
       </c>
-      <c r="I6" s="1" t="inlineStr"/>
-      <c r="J6" s="1" t="inlineStr"/>
-      <c r="K6" s="1" t="inlineStr"/>
-      <c r="L6" s="1" t="inlineStr"/>
-      <c r="M6" s="1" t="inlineStr"/>
-      <c r="N6" s="1" t="inlineStr"/>
     </row>
-    <row r="7" ht="165" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="3" ht="165" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>491</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Pathway 1 - Apply if you're currently employed with a regional NSW employer
 Pathway 2 - Be invited to apply by Investment NSW
 Pathway 3 - Apply if you recently graduated from a Regional NSW institution</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr"/>
-      <c r="E7" s="1" t="inlineStr"/>
-      <c r="F7" s="1" t="inlineStr"/>
-      <c r="G7" s="1" t="inlineStr"/>
-      <c r="H7" s="1" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Timing: Invitation rounds occur throughout the financial year. There are no predetermined or publicly announced dates for invitation rounds.
 Selection: NSW considers multiple factors when selecting EOIs including but not limited to age, English language proficiency, education, points score, and total years of skilled work experience. The highest ranking EOIs within an ANZSCO unit group are invited to apply.
@@ -857,34 +863,61 @@
 The NSW nomination process involves several crucial steps that are different for each nomination pathway:</t>
         </is>
       </c>
-      <c r="I7" s="1" t="inlineStr"/>
-      <c r="J7" s="1" t="inlineStr"/>
-      <c r="K7" s="1" t="inlineStr"/>
-      <c r="L7" s="1" t="inlineStr"/>
-      <c r="M7" s="1" t="inlineStr"/>
-      <c r="N7" s="1" t="inlineStr"/>
     </row>
-    <row r="8" ht="405" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>state code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>state stream</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Detail Requirements</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>service fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="405" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>QLD</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Workers_Living_in_Queensland</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr"/>
-      <c r="D8" s="1" t="inlineStr"/>
-      <c r="E8" s="1" t="inlineStr"/>
-      <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="1" t="inlineStr"/>
-      <c r="H8" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Occupation
 - Have an occupation on the Queensland Onshore Skills List .
@@ -915,34 +948,24 @@
 - Queensland until at least 2 years after the date your Skilled Nominated (Permanent) visa (subclass 190) is granted.</t>
         </is>
       </c>
-      <c r="I8" s="1" t="inlineStr"/>
-      <c r="J8" s="1" t="inlineStr"/>
-      <c r="K8" s="1" t="inlineStr"/>
-      <c r="L8" s="1" t="inlineStr"/>
-      <c r="M8" s="1" t="inlineStr"/>
-      <c r="N8" s="1" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="9" ht="285" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="3" ht="285" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>QLD</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Workers_Living_Offshore</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr"/>
-      <c r="D9" s="1" t="inlineStr"/>
-      <c r="E9" s="1" t="inlineStr"/>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G9" s="1" t="inlineStr"/>
-      <c r="H9" s="1" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Occupation
 - Have an occupation on the Queensland Offshore Skills List .
@@ -965,34 +988,24 @@
 - Queensland until at least 2 years after the date your Skilled Nominated (Permanent) visa (subclass 190) is granted.</t>
         </is>
       </c>
-      <c r="I9" s="1" t="inlineStr"/>
-      <c r="J9" s="1" t="inlineStr"/>
-      <c r="K9" s="1" t="inlineStr"/>
-      <c r="L9" s="1" t="inlineStr"/>
-      <c r="M9" s="1" t="inlineStr"/>
-      <c r="N9" s="1" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="10" ht="360" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="4" ht="360" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>QLD</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Building_and_Construction</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr"/>
-      <c r="D10" s="1" t="inlineStr"/>
-      <c r="E10" s="1" t="inlineStr"/>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G10" s="1" t="inlineStr"/>
-      <c r="H10" s="1" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Occupation
 - Have an occupation on the Queensland Onshore Skills List that is indicated as included in the building and construction workforce pathway.
@@ -1020,34 +1033,24 @@
 - Queensland until at least 2 years after the date your Skilled Nominated (Permanent) visa (subclass 190) is granted.</t>
         </is>
       </c>
-      <c r="I10" s="1" t="inlineStr"/>
-      <c r="J10" s="1" t="inlineStr"/>
-      <c r="K10" s="1" t="inlineStr"/>
-      <c r="L10" s="1" t="inlineStr"/>
-      <c r="M10" s="1" t="inlineStr"/>
-      <c r="N10" s="1" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="11" ht="409" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="5" ht="409" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>QLD</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>University_Graduates</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr"/>
-      <c r="D11" s="1" t="inlineStr"/>
-      <c r="E11" s="1" t="inlineStr"/>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G11" s="1" t="inlineStr"/>
-      <c r="H11" s="1" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Occupation
 Points
@@ -1082,34 +1085,24 @@
 - Queensland until at least 2 years after the date your Skilled Nominated (Permanent) visa (subclass 190) is granted.</t>
         </is>
       </c>
-      <c r="I11" s="1" t="inlineStr"/>
-      <c r="J11" s="1" t="inlineStr"/>
-      <c r="K11" s="1" t="inlineStr"/>
-      <c r="L11" s="1" t="inlineStr"/>
-      <c r="M11" s="1" t="inlineStr"/>
-      <c r="N11" s="1" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="12" ht="120" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="6" ht="120" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>QLD</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Small_Business_Owners</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr"/>
-      <c r="D12" s="1" t="inlineStr"/>
-      <c r="E12" s="1" t="inlineStr"/>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G12" s="1" t="inlineStr"/>
-      <c r="H12" s="1" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Occupation
 - Have an occupation on the Legislative Instrument 19/051 ( LIN19/051 ) .
@@ -1121,34 +1114,24 @@
 - Have evidence you own 100% of the business. 100% ownership is required since the business was purchased or started.</t>
         </is>
       </c>
-      <c r="I12" s="1" t="inlineStr"/>
-      <c r="J12" s="1" t="inlineStr"/>
-      <c r="K12" s="1" t="inlineStr"/>
-      <c r="L12" s="1" t="inlineStr"/>
-      <c r="M12" s="1" t="inlineStr"/>
-      <c r="N12" s="1" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="13" ht="195" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="7" ht="195" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>QLD</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Small_Business_Pathway_1_Purchase</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr"/>
-      <c r="D13" s="1" t="inlineStr"/>
-      <c r="E13" s="1" t="inlineStr"/>
-      <c r="F13" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G13" s="1" t="inlineStr"/>
-      <c r="H13" s="1" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Time since purchase
 - Settlement of business purchase must have occurred less than 18 months before submitting your 491 SBO Registration of Interest.
@@ -1165,68 +1148,90 @@
 - An Australian resident for the purposes of the 491 SBO stream is an Australian citizen, an Australian permanent resident or a New Zealand citizen residing in Australia on a Special Category visa (subclass 444).</t>
         </is>
       </c>
-      <c r="I13" s="1" t="inlineStr"/>
-      <c r="J13" s="1" t="inlineStr"/>
-      <c r="K13" s="1" t="inlineStr"/>
-      <c r="L13" s="1" t="inlineStr"/>
-      <c r="M13" s="1" t="inlineStr"/>
-      <c r="N13" s="1" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>QLD</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Small_Business_Pathway_2_Startup</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr"/>
-      <c r="D14" s="1" t="inlineStr"/>
-      <c r="E14" s="1" t="inlineStr"/>
-      <c r="F14" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G14" s="1" t="inlineStr"/>
-      <c r="H14" s="1" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Requirement
 Operation of business and turnover
 - Have evidence of operating a profitable start-up for a minimum of 2 years, with a turnover of $200,000 in the 12 months prior to submitting your 491 SBO Registration of Interest.</t>
         </is>
       </c>
-      <c r="I14" s="1" t="inlineStr"/>
-      <c r="J14" s="1" t="inlineStr"/>
-      <c r="K14" s="1" t="inlineStr"/>
-      <c r="L14" s="1" t="inlineStr"/>
-      <c r="M14" s="1" t="inlineStr"/>
-      <c r="N14" s="1" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="15" ht="225" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>state code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>state stream</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Detail Requirements</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>service fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="225" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>SA</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Skilled_Employment_in_South_Australia</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr"/>
-      <c r="D15" s="1" t="inlineStr"/>
-      <c r="E15" s="1" t="inlineStr"/>
-      <c r="F15" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G15" s="1" t="inlineStr"/>
-      <c r="H15" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>ELIGIBILITY GUIDELINES
 - Have an active Expression of Interest (EOI) on the Department of Home Affairs' SkillSelect system with South Australia as your first preferred State or Territory.
@@ -1245,34 +1250,24 @@
 - Assessment of employer.</t>
         </is>
       </c>
-      <c r="I15" s="1" t="inlineStr"/>
-      <c r="J15" s="1" t="inlineStr"/>
-      <c r="K15" s="1" t="inlineStr"/>
-      <c r="L15" s="1" t="inlineStr"/>
-      <c r="M15" s="1" t="inlineStr"/>
-      <c r="N15" s="1" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="16" ht="315" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="3" ht="315" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>SA</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>South_Australian_Graduates</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr"/>
-      <c r="D16" s="1" t="inlineStr"/>
-      <c r="E16" s="1" t="inlineStr"/>
-      <c r="F16" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G16" s="1" t="inlineStr"/>
-      <c r="H16" s="1" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>ELIGIBILITY GUIDELINES
 - Have an active Expression of Interest (EOI) on the Department of Home Affairs' SkillSelect system with South Australia as your first preferred State or Territory.
@@ -1297,34 +1292,24 @@
 - Assessment of employer.</t>
         </is>
       </c>
-      <c r="I16" s="1" t="inlineStr"/>
-      <c r="J16" s="1" t="inlineStr"/>
-      <c r="K16" s="1" t="inlineStr"/>
-      <c r="L16" s="1" t="inlineStr"/>
-      <c r="M16" s="1" t="inlineStr"/>
-      <c r="N16" s="1" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="4" ht="150" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>SA</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Outer_Regional_Skilled_Employment</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr"/>
-      <c r="D17" s="1" t="inlineStr"/>
-      <c r="E17" s="1" t="inlineStr"/>
-      <c r="F17" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G17" s="1" t="inlineStr"/>
-      <c r="H17" s="1" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>ELIGIBILITY GUIDELINES
 - Have an active Expression of Interest (EOI) in the Department of Home Affairs SkillSelect system, with South Australia selected as your first preferred state or territory.
@@ -1338,34 +1323,24 @@
 - Your employment must be related to, and at the same skill level as, your nominated occupation. For South Australian nomination, this is generally defined as being within the same Australian and New Zealand Standard Classification of Occupations (ANZSCO) Sub Major Group, represented by the first two digits of the ANZSCO code.</t>
         </is>
       </c>
-      <c r="I17" s="1" t="inlineStr"/>
-      <c r="J17" s="1" t="inlineStr"/>
-      <c r="K17" s="1" t="inlineStr"/>
-      <c r="L17" s="1" t="inlineStr"/>
-      <c r="M17" s="1" t="inlineStr"/>
-      <c r="N17" s="1" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="18" ht="255" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="5" ht="255" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>SA</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Moving_to_South_Australia_from_Overseas</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr"/>
-      <c r="D18" s="1" t="inlineStr"/>
-      <c r="E18" s="1" t="inlineStr"/>
-      <c r="F18" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G18" s="1" t="inlineStr"/>
-      <c r="H18" s="1" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>SUBMIT AN EXPRESSION OF INTEREST (EOI)
  Create an EOI in the SkillSelect system and choose South Australia as your first preferred state or territory.
@@ -1383,31 +1358,76 @@
  If selected, you'll be invited to apply for South Australian state nomination. You will then have 14 days to submit your application, so make sure your EOI details are accurate and up to date.</t>
         </is>
       </c>
-      <c r="I18" s="1" t="inlineStr"/>
-      <c r="J18" s="1" t="inlineStr"/>
-      <c r="K18" s="1" t="inlineStr"/>
-      <c r="L18" s="1" t="inlineStr"/>
-      <c r="M18" s="1" t="inlineStr"/>
-      <c r="N18" s="1" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="19" ht="409" customHeight="1">
-      <c r="A19" s="1" t="inlineStr"/>
-      <c r="B19" s="1" t="inlineStr"/>
-      <c r="C19" s="1" t="inlineStr"/>
-      <c r="D19" s="1" t="inlineStr"/>
-      <c r="E19" s="1" t="inlineStr"/>
-      <c r="F19" s="1" t="inlineStr"/>
-      <c r="G19" s="1" t="inlineStr"/>
-      <c r="H19" s="1" t="inlineStr"/>
-      <c r="I19" s="1" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>state_code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>state_stream</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>tse</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>tsg</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ter</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>tbo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="409" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>TSA</t>
         </is>
       </c>
-      <c r="J19" s="1" t="n">
+      <c r="B2" s="2" t="n">
         <v>190</v>
       </c>
-      <c r="K19" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>[Minimum Requirements]
 You must have worked in Tasmania in a job closely related to your skills assessment (a role within the same ANZSCO 3-digit group as your skills assessment) for:
@@ -1558,7 +1578,7 @@
 Evidence of marriage, dependant relationship if claiming to meet dependant-related priority attributes. Adult dependant must be included in Expression of Interest on SkillSelect.</t>
         </is>
       </c>
-      <c r="L19" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>[Minimum Requirements]
 You must have completed a course with a Tasmanian tertiary institution registered on the Commonwealth Register of Institutions and Courses for Overseas Students (CRICOS) and received a completion letter.
@@ -1721,7 +1741,7 @@
 If they have recently moved to Tasmania from another Australian state or territory, explain what they intend to do in Tasmania.</t>
         </is>
       </c>
-      <c r="M19" s="1" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>[Minimum Requirements]
 be working in a role with a Tasmanian-based employer that paid at least $57,000 per year or $28.85 per hour ( excluding overtime, penalties, bonuses or casual loading ), with at least 12 months of work in the last two years ( minimum 20 hours/week ).
@@ -1874,30 +1894,22 @@
 Evidence of marriage, dependant relationship if claiming to meet dependant-related priority attributes. Adult dependant must be included in Expression of Interest on SkillSelect.</t>
         </is>
       </c>
-      <c r="N19" s="1" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="409" customHeight="1">
-      <c r="A20" s="1" t="inlineStr"/>
-      <c r="B20" s="1" t="inlineStr"/>
-      <c r="C20" s="1" t="inlineStr"/>
-      <c r="D20" s="1" t="inlineStr"/>
-      <c r="E20" s="1" t="inlineStr"/>
-      <c r="F20" s="1" t="inlineStr"/>
-      <c r="G20" s="1" t="inlineStr"/>
-      <c r="H20" s="1" t="inlineStr"/>
-      <c r="I20" s="1" t="inlineStr">
+    <row r="3" ht="409" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>TSA</t>
         </is>
       </c>
-      <c r="J20" s="1" t="n">
+      <c r="B3" s="2" t="n">
         <v>491</v>
       </c>
-      <c r="K20" s="1" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>[Minimum Requirements]
 You must have been working in Tasmania for at least nine months immediately before applying.
@@ -2049,7 +2061,7 @@
 If they have recently moved to Tasmania from another Australian state or territory, explain what they intend to do in Tasmania.</t>
         </is>
       </c>
-      <c r="L20" s="1" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>[Minimum Requirements]
 You must have completed a course with a Tasmanian tertiary institution registered on the Commonwealth Register of Institutions and Courses for Overseas Students (CRICOS) and received a completion letter.
@@ -2214,7 +2226,7 @@
 If they have recently moved to Tasmania from another Australian state or territory, explain what they intend to do in Tasmania.</t>
         </is>
       </c>
-      <c r="M20" s="1" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>[Minimum Requirements]
 be working in a role that paid $57,000 per year or $28.85 per hour ( excluding overtime, penalties, bonuses or casual loading ), with at least 6 months of work in the last year ( minimum 20 hours/week ).
@@ -2351,7 +2363,7 @@
 If they have recently moved to Tasmania from another Australian state or territory, explain what they intend to do in Tasmania.</t>
         </is>
       </c>
-      <c r="N20" s="1" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>[Minimum Requirements]
 You must have established and operated a business in Tasmania for at least 12 months. The business must be solely owned or co-owned with your spouse.
@@ -2471,312 +2483,336 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="409" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>state code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>state stream</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>requirements</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>service fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="409" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>VIC</t>
         </is>
       </c>
-      <c r="B21" s="1" t="inlineStr">
-        <is>
-          <t>Skilled_Nominated_Visa_Subclass_190</t>
-        </is>
-      </c>
-      <c r="C21" s="1" t="inlineStr"/>
-      <c r="D21" s="1" t="inlineStr"/>
-      <c r="E21" s="1" t="inlineStr"/>
-      <c r="F21" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G21" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Subclass_190</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>BASIC ELIGIBILITY
-  To be considered for Victorian skilled visa nomination, you must:
-- meet all the Australian Government's Department of Home Affair’s subclass 190 Skilled Nominated visa requirements.
-- meet all the Victorian Government’s subclass 190 Skilled Nominated visa nomination requirements.
+ To be considered for Victorian skilled visa nomination, you must:
+- meet all the Australian Government's Department of Home Affair's subclass 190 Skilled Nominated visa requirements.
+- meet all the Victorian Government's subclass 190 Skilled Nominated visa nomination requirements.
 VICTORIAN SUBCLASS 190 SKILLED VISA NOMINATION
-  [Who can apply?]
-  To be eligible to apply for Victorian Skilled Nominated (subclass 190) visa nomination, you must:
+ [Who can apply?]
+ To be eligible to apply for Victorian Skilled Nominated (subclass 190) visa nomination, you must:
 - be living in Victoria or overseas,
 - be committed to living and working in Victoria,
 - have had your Registration of Interest (ROI) selected,
 - be under 45 years of age,
 - have at least Competent English, external link
 - have a valid Skills Assessment external link in an occupation on the eligible skilled occupation list external link for this visa,
-- have achieved at least 65 points external link on the Australian Government’s points test for your Expression of Interest (EOI) in SkillSelect.
-  [How to apply?]
-  To apply for Victorian visa nomination, you must:
+- have achieved at least 65 points external link on the Australian Government's points test for your Expression of Interest (EOI) in SkillSelect.
+ [How to apply?]
+ To apply for Victorian visa nomination, you must:
 FURTHER ELIGIBILITY REQUIREMENTS
-  [Living in Victoria]
-  If you are living in Australia (onshore) you must be living in Victoria . We will not be selecting Registration of Interests (ROIs) from onshore applicants living in Australian states and territories other than Victoria. We do make some case-by-case exceptions for those living in border communities.
-  [Living overseas]
-  If you are living overseas (offshore), you are eligible to apply for Skilled Nominated (subclass 190) visa nomination. You must be committed to living in Victoria.
-  [Employment]
-  You are not required to be working to be eligible for Victorian subclass 190 visa nomination. There is no minimum work experience and hours of work requirement.
-  Living in Victoria (onshore):
+ [Living in Victoria]
+ If you are living in Australia (onshore) you must be living in Victoria . We will not be selecting Registration of Interests (ROIs) from onshore applicants living in Australian states and territories other than Victoria. We do make some case-by-case exceptions for those living in border communities.
+ [Living overseas]
+ If you are living overseas (offshore), you are eligible to apply for Skilled Nominated (subclass 190) visa nomination. You must be committed to living in Victoria.
+ [Employment]
+ You are not required to be working to be eligible for Victorian subclass 190 visa nomination. There is no minimum work experience and hours of work requirement.
+ Living in Victoria (onshore):
 - If you are living in Victoria and work in skilled employment for an employer physically located in Victoria , you can provide an estimate of your annual earnings in your ROI . A business using a virtual office or proxy office is not considered as physically located in Victoria. Your employment does not have to be related to or the same as your nominated occupation, but your earnings must be from skilled employment in Victoria. View our Annual earnings estimation guide for information on skilled employment and what you can and cannot claim.
 - If you are not working, working in non-skilled employment, or working for an employer not physically located in Victoria, you are still eligible to apply for nomination, but you are not eligible to claim earnings in your ROI.
-  Living overseas (offshore):
+ Living overseas (offshore):
 - If you are living overseas, you are not required to claim earnings in your ROI.
-  [Commitment to Victoria]
+ [Commitment to Victoria]
 - You must be committed to living and working in Victoria.
 - State nomination cannot be transferred from one state to another.
-  [Registration of Interest]
+ [Registration of Interest]
 - To be invited to apply for Victorian visa nomination, you must submit an ROI.
 - Your ROI must be selected by us before you can apply for skilled visa nomination. An ROI is not an application for Victorian visa nomination. There is no guarantee that your ROI will be selected.
 - View our Registration of Interest page for more information on assessment and selection considerations.
-  [Age]
+ [Age]
 - You must be under 45 years of age at the time of nomination. This is a Department of Home Affairs requirement.
-  [English language]
+ [English language]
 - You must have at least Competent English external link .
 - When you submit your nomination application, we require that your English test has at least 12 weeks validity remaining. This ensures we have enough time to assess your nomination application. We cannot nominate you if your English test has expired.
-- For further information, see the Australian Government's Department of Home Affairs’ English language requirements external link page.
-  [Skills Assessment]
-- You must have a valid skills assessment in an occupation on the Australian Government’s eligible skilled occupation list external link for the visa.
+- For further information, see the Australian Government's Department of Home Affairs' English language requirements external link page.
+ [Skills Assessment]
+- You must have a valid skills assessment in an occupation on the Australian Government's eligible skilled occupation list external link for the visa.
 - Your nominated occupation in your Skills Assessment external link must match your SkillSelect Expression of Interest (EOI) with the Department of Home Affairs.
 - When you submit your nomination application, we require that your Skills Assessment external link has at least 12 weeks validity remaining. This ensures we have enough time to assess your nomination application. We cannot nominate you if your Skills Assessment has expired.
-- For Health professionals, your occupation must be consistent with your Australian Health Practitioner Regulation Agency (AHPRA) registration.
-  [SkillSelect EOI Points]
-- You must have at least 65 points on the Australian Government’s points test external link , including the 5 points for state and territory nomination.
+- For Health professionals, your occupation must be consistent with your Australian Health Practitioner Regulation Agency (AHPRA) registration.
+ [SkillSelect EOI Points]
+- You must have at least 65 points on the Australian Government's points test external link , including the 5 points for state and territory nomination.
 INVITATION TO APPLY FOR VICTORIAN NOMINATION
-  To be invited to apply for Victorian skilled visa nomination, you must firstly make or update an Expression of Interest via the Australian Government’s SkillSelect external link and then submit a Registration of Interest (ROI).
-  View our Registration of Interest page for more information on ROI assessment and selection considerations.
-  For information on how to calculate your estimated annual earnings, visit our Annual Earnings Estimation Guide page. Answers to frequently asked questions can be found on our Skilled Visa FAQs page.
+ To be invited to apply for Victorian skilled visa nomination, you must firstly make or update an Expression of Interest via the Australian Government's SkillSelect external link and then submit a Registration of Interest (ROI).
+ View our Registration of Interest page for more information on ROI assessment and selection considerations.
+ For information on how to calculate your estimated annual earnings, visit our Annual Earnings Estimation Guide page. Answers to frequently asked questions can be found on our Skilled Visa FAQs page.
 SUBMITTING A NOMINATION APPLICATION
-  [Submit your application via the portal]
-  If you are invited to apply, you or your agent (if applicable) will be notified via email.
-  You must submit your application and all documents via the Live in Melbourne portal external link . We will not accept any applications or documents via email.
-  [What documents you will need]
-  If you are invited to apply for Victorian nomination, you must submit a complete application, including all relevant evidence to support your eligibility claims.
-  In your Victorian nomination application, you may need to provide the following documents to show you meet the requirements:
+ [Submit your application via the portal]
+ If you are invited to apply, you or your agent (if applicable) will be notified via email.
+ You must submit your application and all documents via the Live in Melbourne portal external link . We will not accept any applications or documents via email.
+ [What documents you will need]
+ If you are invited to apply for Victorian nomination, you must submit a complete application, including all relevant evidence to support your eligibility claims.
+ In your Victorian nomination application, you may need to provide the following documents to show you meet the requirements:
 - passport,
 - evidence of Victorian residence.
-  During the assessment of your nomination application, we may ask for further evidence and additional documents.
-  [Living in Victoria:]
-  To prove your residence in Victoria, you may be asked to provide the following documents to show you meet the requirements:
+ During the assessment of your nomination application, we may ask for further evidence and additional documents.
+ [Living in Victoria:]
+ To prove your residence in Victoria, you may be asked to provide the following documents to show you meet the requirements:
 - bank statements for a minimum of 6 months from your main transaction account showing your salary and everyday transactions,
 - rental or lease agreements,
 - utility bills e.g. gas, water, phone, internet,
-- driver’s licence or proof of age cards.
-  If you included annual earnings in your Registration of Interest (ROI) you will also need to provide the following in your nomination application:
+- driver's licence or proof of age cards.
+ If you included annual earnings in your Registration of Interest (ROI) you will also need to provide the following in your nomination application:
 - employment contract,
 - position description detailing the duration of your employment, the hours worked per week, and duties performed,
 - payslips (at least most recent four weeks),
 - superannuation statement (showing most recent contributions), or
 - your letter of offer.
 NOMINATION APPLICATION ASSESSMENT
-  If you submit a nomination application, it will be assessed by the Victorian Government. You will be notified of the outcome by email as soon as a decision has been made.
-  [Respond within two weeks]
-  We may ask you for more information by email.
+ If you submit a nomination application, it will be assessed by the Victorian Government. You will be notified of the outcome by email as soon as a decision has been made.
+ [Respond within two weeks]
+ We may ask you for more information by email.
 - You will have two weeks to provide the requested information.
 - If you do not respond within two weeks, we may refuse your application. Please check your junk mail and ensure the email address no-reply-gems@liveinmelbourne.vic.gov.au external link is added to your list of valid email addresses.
-  [Incomplete applications]
-  You must submit a complete application, including all relevant evidence to support your eligibility claims.
-  [Do not ask for updates on your application]
-  Please do not ask for an update on your application. We assess all applications in order of when they are submitted.
-  If you have submitted a nomination application with us, you or your agent (if applicable) can check the status of your application through the Live in Melbourne portal. The average processing time for skilled visa nomination applications is 20 business days. This does not include the waiting time if we require additional information for your application.
-  The assessment team is also responsible for responding to enquiries and we prioritise assessment of applications. Unnecessary enquiries slow down application processing times.
-  [Withdrawal]
-  You can only withdraw your subclass 190 nomination application before we finalise our assessment. Please Contact Us to withdraw your nomination application.
-  For Registrations of Interest (ROIs), you must withdraw your ROI using the Live in Melbourne portal. external link
+ [Incomplete applications]
+ You must submit a complete application, including all relevant evidence to support your eligibility claims.
+ [Do not ask for updates on your application]
+ Please do not ask for an update on your application. We assess all applications in order of when they are submitted.
+ If you have submitted a nomination application with us, you or your agent (if applicable) can check the status of your application through the Live in Melbourne portal. The average processing time for skilled visa nomination applications is 20 business days. This does not include the waiting time if we require additional information for your application.
+ The assessment team is also responsible for responding to enquiries and we prioritise assessment of applications. Unnecessary enquiries slow down application processing times.
+ [Withdrawal]
+ You can only withdraw your subclass 190 nomination application before we finalise our assessment. Please Contact Us to withdraw your nomination application.
+ For Registrations of Interest (ROIs), you must withdraw your ROI using the Live in Melbourne portal. external link
 NOMINATION APPLICATION OUTCOME
-  [Once you are nominated]
-  [Nomination refusals]
-  Before submitting a Registration of Interest (ROI) make sure you meet all the minimum eligibility requirements for the visa you are seeking nomination for.
-  Your nomination application will be refused for the following reasons:
+ [Once you are nominated]
+ [Nomination refusals]
+ Before submitting a Registration of Interest (ROI) make sure you meet all the minimum eligibility requirements for the visa you are seeking nomination for.
+ Your nomination application will be refused for the following reasons:
 - You do not meet the minimum eligibility requirements.
 - You cannot provide sufficient evidence for the claims made in your ROI or SkillSelect EOI.
 - You do not respond to our requests for further information in a timely manner.
 - You provide false or misleading information.
-  Common reasons for refused applications include:
+ Common reasons for refused applications include:
 - Over-estimated earnings (for onshore).
 - Working in employment that is not eligible (for onshore).
 - Working for an employer not operating in Victoria (for onshore).
 - Living in an Australian state and territory other than Victoria (for onshore)
 - Incorrect partner points.
-- Modification of SkillSelect EOI after invitation.
+- Modification of SkillSelect EOI after invitation.
 - False and misleading information related to employment and residence.
 - Expired Skills Assessment or English language test results.
-  If you are unable to provide sufficient evidence to demonstrate the claims you make in your SkillSelect EOI and ROI, your application may be refused.
-  If your application is refused, you will not be able to submit a new application for 6 months. This ensures our resources are allocated to processing applications that meet the requirements of the visa.
-  [False and misleading information]
-  If you provide false or misleading information as part of your nomination application, your application will be refused. We may also report it to the Department of Home Affairs who can conduct their own investigation.
-  We encourage you to submit all documents unaltered, including all PDF documents in their original form and not combined into one document.
-  We conduct verification checks on many of the documents you provide to ensure that your employment matches the skill level of your nominated occupation that you outline in your SkillSelect EOI. This includes contacting employers and institutions directly to confirm whether the documents are genuine.
-  If you are aware of instances, or yourself are pressured to submit an application with false and misleading information, we encourage you to report this to the Department of Home Affairs.
-  [Review of nomination decision]
-  If your nomination application has been refused as you did not meet the eligibility requirements, you cannot request a review of your application.
-  If you believe that an error was made in assessing your nomination application, you can submit a request for us to review the application.
-  [Renomination]
-  We do not provide renomination in the following instances:
+ If you are unable to provide sufficient evidence to demonstrate the claims you make in your SkillSelect EOI and ROI, your application may be refused.
+ If your application is refused, you will not be able to submit a new application for 6 months. This ensures our resources are allocated to processing applications that meet the requirements of the visa.
+ [False and misleading information]
+ If you provide false or misleading information as part of your nomination application, your application will be refused. We may also report it to the Department of Home Affairs who can conduct their own investigation.
+ We encourage you to submit all documents unaltered, including all PDF documents in their original form and not combined into one document.
+ We conduct verification checks on many of the documents you provide to ensure that your employment matches the skill level of your nominated occupation that you outline in your SkillSelect EOI. This includes contacting employers and institutions directly to confirm whether the documents are genuine.
+ If you are aware of instances, or yourself are pressured to submit an application with false and misleading information, we encourage you to report this to the Department of Home Affairs.
+ [Review of nomination decision]
+ If your nomination application has been refused as you did not meet the eligibility requirements, you cannot request a review of your application.
+ If you believe that an error was made in assessing your nomination application, you can submit a request for us to review the application.
+ [Renomination]
+ We do not provide renomination in the following instances:
 - You do not submit your visa application within 60 days.
 - Your SkillSelect EOI was incorrect when we nominated you, including points claimed by you or your agent.
-  If an applicant has been nominated for any skilled subclass (either 190 or 491), they cannot be nominated again in the same program year.
+ If an applicant has been nominated for any skilled subclass (either 190 or 491), they cannot be nominated again in the same program year.
 YOUR NOMINATION OBLIGATIONS
-  [Declaration form]
-  If you are nominated, you must meet the nomination obligations that you signed in the declaration form .
-  [Surveys]
-  If you are nominated, we will contact you at various times.
-  In the declaration form, you agree to complete surveys if requested by, or on behalf of the Victorian Government, including a survey upon arrival and at six monthly intervals for the two years after visa grant or arrival in Australia.
-  These surveys are a condition of nomination. They provide us important feedback on our client services and policy settings. The surveys do not have an impact on your visa.
-  [Department of Home Affairs and SkillSelect]
-  The Australian Government's Department of Home Affairs external link is responsible for all visa matters. This includes once you have been nominated by the Victorian Government and have submitted your visa application.
-  Please check subclass 190 visa processing times external link published by the Department of Home Affairs.
-  All SkillSelect and Expressions of Interest (EOI) enquiries should be directed to the Department of Home Affairs.
+ [Declaration form]
+ If you are nominated, you must meet the nomination obligations that you signed in the declaration form .
+ [Surveys]
+ If you are nominated, we will contact you at various times.
+ In the declaration form, you agree to complete surveys if requested by, or on behalf of the Victorian Government, including a survey upon arrival and at six monthly intervals for the two years after visa grant or arrival in Australia.
+ These surveys are a condition of nomination. They provide us important feedback on our client services and policy settings. The surveys do not have an impact on your visa.
+ [Department of Home Affairs and SkillSelect]
+ The Australian Government's Department of Home Affairs external link is responsible for all visa matters. This includes once you have been nominated by the Victorian Government and have submitted your visa application.
+ Please check subclass 190 visa processing times external link published by the Department of Home Affairs.
+ All SkillSelect and Expressions of Interest (EOI) enquiries should be directed to the Department of Home Affairs.
 TERMS AND CONDITIONS
-  [Can my employer or family member represent me as an agent for Victorian nomination?]
-  No, you cannot appoint an agent to act on your behalf if there are personal, financial or other interests that could, or could be seen to, influence their representation of you.
-  If a conflict of interest is identified during the application assessment, the Appointment of Agent will be deemed invalid, and the application may be refused.
-  [Nomination application fees]
-  Victorian Registration of Interest (ROI) and nomination are free of charge. When you submit your visa application with the Australian Government's Department of Home Affairs, you will need to pay the visa fee.
-  [Changes to eligibility requirements]
-  All visa nomination eligibility requirements and priorities are subject to change throughout the year without notice.
-  Any changes made are effective immediately, regardless of when your SkillSelect Expression of Interest (EOI) was submitted (or amended). We strongly discourage changing your circumstances to meet the visa nomination criteria.
-  The Victorian Government endeavours to ensure all information on the Live in Melbourne website reflects the current eligibility requirements. The Live in Melbourne website is the authoritative source for information about Victoria's skilled visa nomination program.</t>
-        </is>
-      </c>
-      <c r="H21" s="1" t="inlineStr"/>
-      <c r="I21" s="1" t="inlineStr"/>
-      <c r="J21" s="1" t="inlineStr"/>
-      <c r="K21" s="1" t="inlineStr"/>
-      <c r="L21" s="1" t="inlineStr"/>
-      <c r="M21" s="1" t="inlineStr"/>
-      <c r="N21" s="1" t="inlineStr"/>
+ [Can my employer or family member represent me as an agent for Victorian nomination?]
+ No, you cannot appoint an agent to act on your behalf if there are personal, financial or other interests that could, or could be seen to, influence their representation of you.
+ If a conflict of interest is identified during the application assessment, the Appointment of Agent will be deemed invalid, and the application may be refused.
+ [Nomination application fees]
+ Victorian Registration of Interest (ROI) and nomination are free of charge. When you submit your visa application with the Australian Government's Department of Home Affairs, you will need to pay the visa fee.
+ [Changes to eligibility requirements]
+ All visa nomination eligibility requirements and priorities are subject to change throughout the year without notice.
+ Any changes made are effective immediately, regardless of when your SkillSelect Expression of Interest (EOI) was submitted (or amended). We strongly discourage changing your circumstances to meet the visa nomination criteria.
+ The Victorian Government endeavours to ensure all information on the Live in Melbourne website reflects the current eligibility requirements. The Live in Melbourne website is the authoritative source for information about Victoria's skilled visa nomination program.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="22" ht="409" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
+    <row r="3" ht="409" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>VIC</t>
         </is>
       </c>
-      <c r="B22" s="1" t="inlineStr">
-        <is>
-          <t>Skilled_Work_Regional_Visa_Subclass_491</t>
-        </is>
-      </c>
-      <c r="C22" s="1" t="inlineStr"/>
-      <c r="D22" s="1" t="inlineStr"/>
-      <c r="E22" s="1" t="inlineStr"/>
-      <c r="F22" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G22" s="1" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Subclass_491</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>BASIC ELIGIBILITY
-  To be considered for Victorian skilled visa nomination, you must:
+ To be considered for Victorian skilled visa nomination, you must:
 - Meet all the Department of Home Affairs - subclass 491 Skilled Work Regional (Provisional) visa requirements external link .
-- Meet all the Victorian Government’s - subclass 491Skilled Nominated visa requirements.
+- Meet all the Victorian Government's - subclass 491Skilled Nominated visa requirements.
 VICTORIAN SUBCLASS 491 SKILLED WORK REGIONAL VISA NOMINATION
-  [Who can apply?]
-  To be eligible to apply for Skilled Work Regional (Provisional) visa (subclass 491) nomination, you must:
+ [Who can apply?]
+ To be eligible to apply for Skilled Work Regional (Provisional) visa (subclass 491) nomination, you must:
 - be one of the following: living offshore living and working in regional Victoria.
 - be committed to living and working in regional Victoria,
 - have had your Registration of Interest (ROI) selected,
 - be under 45 years of age,
 - have at least Competent English external link ,
 - have a valid skills assessment external link in an occupation on the eligible skilled occupation list external link for this visa,
-- have achieved at least 65 points external link on the Australian Government’s points test for your Expression of Interest (EOI) in SkillSelect external link .
+- have achieved at least 65 points external link on the Australian Government's points test for your Expression of Interest (EOI) in SkillSelect external link .
 - living offshore
 - living and working in regional Victoria.
-  [How to apply?]
-  To apply for Victorian visa nomination, you must:
+ [How to apply?]
+ To apply for Victorian visa nomination, you must:
 FURTHER ELIGIBILITY REQUIREMENTS
-  [Living overseas]
-  Residence
-  If you are living overseas (offshore), you are eligible to apply for Skilled Work Regional (Provisional) visa (subclass 491) visa nomination.
-  Once you are granted the subclass 491 visa you will be required to relocate to regional Victoria. The conditions of the subclass 491 visa require you, and any dependent applicants, to live, work, and study in a designated regional area.
-  Employment
-  If you are living overseas, you are not required to claim earnings in your ROI .
-  [Living in Victoria]
-  Residence
-  You must be living in regional Victoria external link .
-- Some outer suburbs of Melbourne are considered regional for the purposes of migration by the Australian's Government's Department of Home Affairs. For example, the Mornington Peninsula, Pakenham and Geelong are considered designated regional areas of Victoria for migration purposes.
+ [Living overseas]
+ Residence
+ If you are living overseas (offshore), you are eligible to apply for Skilled Work Regional (Provisional) visa (subclass 491) visa nomination.
+ Once you are granted the subclass 491 visa you will be required to relocate to regional Victoria. The conditions of the subclass 491 visa require you, and any dependent applicants, to live, work, and study in a designated regional area.
+ Employment
+ If you are living overseas, you are not required to claim earnings in your ROI .
+ [Living in Victoria]
+ Residence
+ You must be living in regional Victoria external link .
+- Some outer suburbs of Melbourne are considered regional for the purposes of migration by the Australian's Government's Department of Home Affairs. For example, the Mornington Peninsula, Pakenham and Geelong are considered designated regional areas of Victoria for migration purposes.
 - You can find information about the designated regional areas external link on the Department of Home Affairs website.
 - We make case-by-case exceptions for those living in border communities.
-  The conditions of the subclass 491 visa require you, and any dependent applicants, to live, work, and study in a designated regional area.
-  Employment
-- You must be working in skilled employment for an employer physically located in regional Victoria. A business using a virtual office or proxy office is not considered as physically located in regional Victoria.
+ The conditions of the subclass 491 visa require you, and any dependent applicants, to live, work, and study in a designated regional area.
+ Employment
+- You must be working in skilled employment for an employer physically located in regional Victoria. A business using a virtual office or proxy office is not considered as physically located in regional Victoria.
 - A business using a virtual office or proxy office is not considered as physically located in regional Victoria.
-- You must provide an estimate of your annual earnings in your ROI . Your earnings must be from skilled employment in regional Victoria. View our Annual earnings estimation guide for information on skilled employment and what you can and cannot claim.
+- You must provide an estimate of your annual earnings in your ROI . Your earnings must be from skilled employment in regional Victoria. View our Annual earnings estimation guide for information on skilled employment and what you can and cannot claim.
 - View our Annual earnings estimation guide for information on skilled employment and what you can and cannot claim.
 - Your employment does not have to be related to or the same as your nominated occupation.
 - There is no minimum requirement for hours worked.
 - If you are not working, working in non-skilled employment, or working for an employer who is not physically located in regional Victoria, you are not eligible to apply for nomination.
-  [Commitment to regional Victoria]
+ [Commitment to regional Victoria]
 - You must be committed to living and working in a designated regional area of Victoria external link .
 - State nomination cannot be transferred from one state to another.
-  [Registration of Interest]
+ [Registration of Interest]
 - To be invited to apply for Victorian visa nomination, you must submit an ROI.
 - Your ROI must be selected by us before you can apply for skilled visa nomination. An ROI is not an application for Victorian visa nomination. There is no guarantee that your ROI will be selected.
 - View our Registration of Interest page for more information on assessment and selection considerations.
-  [Age]
+ [Age]
 - You must be under 45 years of age at the time of nomination. This is a Department of Home Affairs requirement.
-  [English language]
+ [English language]
 - You must have at least Competent English external link .
 - When you submit your nomination application, we require that your English language test has at least 12 weeks validity remaining. This ensures we have enough time to assess your nomination application. We cannot nominate you if your English language test has expired.
 - For further information, see the Australian Government's Department of Home Affairs English language requirements external link page.
-  [Skills Assessment]
+ [Skills Assessment]
 - You must have a valid skills assessment in an occupation on the eligible skilled occupation list external link for the visa.
 - Your nominated occupation in your Skills Assessment external link must match your Expression of Interest with the Department of Home Affairs.
 - When you submit your nomination application, we require that your Skills Assessment has at least 12 weeks validity remaining. This ensures we have enough time to assess your nomination application. We cannot nominate you if your Skills Assessment has expired.
-- For Health professionals, your occupation must be consistent with your Australian Health Practitioner Regulation Agency (AHPRA) registration.
-  [SkillSelect EOI Points]
-- You must have at least 65 points external link on the Australian Government’s points test external link , including the 15 points for state and territory nomination.
+- For Health professionals, your occupation must be consistent with your Australian Health Practitioner Regulation Agency (AHPRA) registration.
+ [SkillSelect EOI Points]
+- You must have at least 65 points external link on the Australian Government's points test external link , including the 15 points for state and territory nomination.
 INVITATION TO APPLY FOR VICTORIAN NOMINATION
-  To be invited to apply for Victorian skilled visa nomination, you must firstly submit or update an Expression of Interest via the Australian Government’s SkillSelect and then submit a Registration of Interest (ROI).
-  View our Registration of Interest page for more information on ROI assessment and selection considerations.
-  For information on how to calculate your estimated annual earnings, visit our Annual Earnings Estimation Guide page. Answers to frequently asked questions can be found on our Skilled Visa FAQs page.
+ To be invited to apply for Victorian skilled visa nomination, you must firstly submit or update an Expression of Interest via the Australian Government's SkillSelect and then submit a Registration of Interest (ROI).
+ View our Registration of Interest page for more information on ROI assessment and selection considerations.
+ For information on how to calculate your estimated annual earnings, visit our Annual Earnings Estimation Guide page. Answers to frequently asked questions can be found on our Skilled Visa FAQs page.
 SUBMITTING A NOMINATION APPLICATION
-  [Submit your application via the portal]
-  If you are invited to apply, you or your agent (if applicable) will be notified via email.
-  You must submit your application and all documents via the Live in Melbourne portal external link . We will not accept any applications or documents via email.
-  [What documents you will need]
-  If you are invited to apply for Victorian nomination, you must submit a complete application, including all relevant evidence to support your eligibility claims.
-  In your Victorian nomination application, you may need to provide the following documents to show you meet the requirements:
+ [Submit your application via the portal]
+ If you are invited to apply, you or your agent (if applicable) will be notified via email.
+ You must submit your application and all documents via the Live in Melbourne portal external link . We will not accept any applications or documents via email.
+ [What documents you will need]
+ If you are invited to apply for Victorian nomination, you must submit a complete application, including all relevant evidence to support your eligibility claims.
+ In your Victorian nomination application, you may need to provide the following documents to show you meet the requirements:
 - passport,
 - evidence of Victorian residence.
-  During the assessment of your nomination application, we may ask for further evidence and additional documents.
-  Living in regional Victoria:
-  To prove your residence in regional Victoria, you may be asked to provide the following documents to show you meet the requirements:
+ During the assessment of your nomination application, we may ask for further evidence and additional documents.
+ Living in regional Victoria:
+ To prove your residence in regional Victoria, you may be asked to provide the following documents to show you meet the requirements:
 - bank statements for a minimum of 6 months from your main transaction account showing your salary and everyday transactions,
 - rental or lease agreements,
 - utility bills e.g. gas, water, phone, internet,
-- driver’s licence or proof of age cards.
-  If you included annual earnings in your Registration of Interest (ROI) you will also need to provide the following in your nomination application:
+- driver's licence or proof of age cards.
+ If you included annual earnings in your Registration of Interest (ROI) you will also need to provide the following in your nomination application:
 - employment contract,
 - position description detailing the duration of your employment, the hours worked per week and duties performed
 - payslips (at least most recent four weeks),
 - superannuation statement (showing most recent contributions),
 - your letter of offer.
 NOMINATION APPLICATION ASSESSMENT
-  Following submission of your nomination application, you will be notified of the outcome by email as soon as a decision has been made.
-  [Respond within two weeks]
-  We may ask you for more information by email.
+ Following submission of your nomination application, you will be notified of the outcome by email as soon as a decision has been made.
+ [Respond within two weeks]
+ We may ask you for more information by email.
 - You will have two weeks to provide the requested information.
 - If you do not respond within two weeks, we may refuse your application. Please check your junk mail and ensure the email address no-reply-gems@liveinmelbourne.vic.gov.au external link is added to your list of valid email addresses.‎‎‎
-  [Incomplete applications]
-  You must submit a complete application, including all relevant evidence to support your eligibility claims.
-  [Please do not ask for updates on your application]
-  Please do not ask for an update on your application. We assess all applications in order of when they are submitted.
-  If you have submitted a nomination application, you or your agent (if applicable) can check the status of your application through the Live in Melbourne portal. external link The average processing time for skilled visa nomination applications is 20 business days. This does not include the waiting time if we require additional information for your application.
-  The assessment team is also responsible for responding to enquiries and we prioritise assessment of applications. Unnecessary enquiries slow down application processing times.
-  [Withdrawal]
-  You can only withdraw your subclass 491 nomination application before we finalise our assessment. Please Contact Us to withdraw your nomination application.
-  For Registrations of Interest (ROI), you must withdraw your ROI using the Live in Melbourne portal external link .
+ [Incomplete applications]
+ You must submit a complete application, including all relevant evidence to support your eligibility claims.
+ [Please do not ask for updates on your application]
+ Please do not ask for an update on your application. We assess all applications in order of when they are submitted.
+ If you have submitted a nomination application, you or your agent (if applicable) can check the status of your application through the Live in Melbourne portal. external link The average processing time for skilled visa nomination applications is 20 business days. This does not include the waiting time if we require additional information for your application.
+ The assessment team is also responsible for responding to enquiries and we prioritise assessment of applications. Unnecessary enquiries slow down application processing times.
+ [Withdrawal]
+ You can only withdraw your subclass 491 nomination application before we finalise our assessment. Please Contact Us to withdraw your nomination application.
+ For Registrations of Interest (ROI), you must withdraw your ROI using the Live in Melbourne portal external link .
 NOMINATION APPLICATION OUTCOME
-  [Once you are nominated]
-  [Nomination refusals]
-  Before submitting a Registration of Interest (ROI) make sure you meet all the minimum eligibility requirements for the visa you are seeking nomination for.
-  Your nomination application will be refused for the following reasons:
+ [Once you are nominated]
+ [Nomination refusals]
+ Before submitting a Registration of Interest (ROI) make sure you meet all the minimum eligibility requirements for the visa you are seeking nomination for.
+ Your nomination application will be refused for the following reasons:
 - You do not meet the minimum eligibility requirements.
 - You cannot provide sufficient evidence for the claims made in your ROI or SkillSelect EOI.
 - You provide false or misleading information.
 - You do not respond to our requests for further information in a timely manner.
-  Common reasons for refused applications include:
+ Common reasons for refused applications include:
 - Over-estimated earnings (for onshore).
 - Working in a non-skilled employment (for onshore).
 - Working for an employer not operating in regional Victoria (for onshore).
@@ -2785,72 +2821,104 @@
 - Modification of your SkillSelect EOI after invitation.
 - Integrity concerns with residence and employment claims.
 - Skills assessment or English language test result expired.
-  If you are unable to provide sufficient evidence to demonstrate the claims you make in your SkillSelect EOI and ROI, your application may be refused.
-  If your application is refused, you will not be able to submit a new application for 6 months. This ensures our resources are allocated to processing applications that meet the requirements of the visa.
-  [False and misleading information]
-  If you provide false or misleading information as part of your nomination application, your application will be refused. We may also report it to the Department of Home Affairs who can conduct their own investigation.
-  We encourage you to submit all documents unaltered, including all PDF documents in their original form and not combined into one document.
-  We conduct verification checks on many of the documents you provide to ensure that your employment matches the skill level of your nominated occupation that you outline in your SkillSelect EOI. This includes contacting employers and institutions directly to confirm whether the documents are genuine.
-  If you are aware of instances, or yourself are pressured to submit an application with false and misleading information, we encourage you to report this to the Department of Home Affairs.
-  [Review of nomination decision]
-  If your nomination application has been refused as you did not meet the eligibility requirements, you cannot request a review of your application.
-  If you believe that an error was made in assessing your nomination application, you can submit a request for us to review the application.
-  [Renomination]
-  We do not provide renomination in the following instances:
+ If you are unable to provide sufficient evidence to demonstrate the claims you make in your SkillSelect EOI and ROI, your application may be refused.
+ If your application is refused, you will not be able to submit a new application for 6 months. This ensures our resources are allocated to processing applications that meet the requirements of the visa.
+ [False and misleading information]
+ If you provide false or misleading information as part of your nomination application, your application will be refused. We may also report it to the Department of Home Affairs who can conduct their own investigation.
+ We encourage you to submit all documents unaltered, including all PDF documents in their original form and not combined into one document.
+ We conduct verification checks on many of the documents you provide to ensure that your employment matches the skill level of your nominated occupation that you outline in your SkillSelect EOI. This includes contacting employers and institutions directly to confirm whether the documents are genuine.
+ If you are aware of instances, or yourself are pressured to submit an application with false and misleading information, we encourage you to report this to the Department of Home Affairs.
+ [Review of nomination decision]
+ If your nomination application has been refused as you did not meet the eligibility requirements, you cannot request a review of your application.
+ If you believe that an error was made in assessing your nomination application, you can submit a request for us to review the application.
+ [Renomination]
+ We do not provide renomination in the following instances:
 - You do not submit your visa application within 60 days.
 - Your SkillSelect EOI was incorrect when we nominated you, including points claimed by you or your agent.
-  If an applicant has been nominated for any skilled visa (either subclass 190 or 491), they cannot be nominated again in the same program year.
+ If an applicant has been nominated for any skilled visa (either subclass 190 or 491), they cannot be nominated again in the same program year.
 YOUR NOMINATION OBLIGATIONS
-  [Declaration form]
-  If you are nominated, you must meet the nomination obligations that you signed in the declaration form .
-  [Surveys]
-  If you are nominated, we will contact you at various times.
-  In the declaration form, you agree to complete surveys if requested by, or on behalf of the Victorian Government, including a survey upon arrival and at six monthly intervals for the three years after visa grant or arrival in Australia.
-  These surveys are a condition of nomination. They provide us important feedback on our client services and policy settings.
-  [Department of Home Affairs and SkillSelect]
-  The Australian Government's Department of Home Affairs external link is responsible for all visa matters. This includes once you have been nominated by the Victorian Government and have submitted your visa application.
-  Please check subclass 491 visa processing times external link published by the Department of Home Affairs.
-  All SkillSelect and Expression of Interest enquiries should be directed to the Department of Home Affairs .
+ [Declaration form]
+ If you are nominated, you must meet the nomination obligations that you signed in the declaration form .
+ [Surveys]
+ If you are nominated, we will contact you at various times.
+ In the declaration form, you agree to complete surveys if requested by, or on behalf of the Victorian Government, including a survey upon arrival and at six monthly intervals for the three years after visa grant or arrival in Australia.
+ These surveys are a condition of nomination. They provide us important feedback on our client services and policy settings.
+ [Department of Home Affairs and SkillSelect]
+ The Australian Government's Department of Home Affairs external link is responsible for all visa matters. This includes once you have been nominated by the Victorian Government and have submitted your visa application.
+ Please check subclass 491 visa processing times external link published by the Department of Home Affairs.
+ All SkillSelect and Expression of Interest enquiries should be directed to the Department of Home Affairs .
 TERMS AND CONDITIONS
-  [Can my employer or family member represent me as an agent for Victorian nomination?]
-  No, you cannot appoint an agent to act on your behalf if there are personal, financial or other interests that could, or could be seen to, influence their representation of you.
-  If a conflict of interest is identified during the application assessment, the Appointment of Agent will be deemed invalid, and the application may be refused.
-  [Nomination application fees]
-  Victorian Registration of Interest (ROI) and nomination are free of charge. When you submit your visa application with the Australian Government's Department of Home Affairs, you will need to pay the visa fee.
-  [Changes to eligibility requirements]
-  All visa nomination eligibility requirements and priorities are subject to change throughout the year without notice.
-  Any changes made are effective immediately, regardless of when your SkillSelect Expression of Interest (EOI) was submitted (or amended). We strongly discourage changing your circumstances to meet the visa nomination criteria.
-  The Victorian Government endeavours to ensure all information on the Live in Melbourne website reflects the current eligibility requirements. The Live in Melbourne website is the authoritative source for information about Victoria's skilled visa nomination program.</t>
-        </is>
-      </c>
-      <c r="H22" s="1" t="inlineStr"/>
-      <c r="I22" s="1" t="inlineStr"/>
-      <c r="J22" s="1" t="inlineStr"/>
-      <c r="K22" s="1" t="inlineStr"/>
-      <c r="L22" s="1" t="inlineStr"/>
-      <c r="M22" s="1" t="inlineStr"/>
-      <c r="N22" s="1" t="inlineStr"/>
+ [Can my employer or family member represent me as an agent for Victorian nomination?]
+ No, you cannot appoint an agent to act on your behalf if there are personal, financial or other interests that could, or could be seen to, influence their representation of you.
+ If a conflict of interest is identified during the application assessment, the Appointment of Agent will be deemed invalid, and the application may be refused.
+ [Nomination application fees]
+ Victorian Registration of Interest (ROI) and nomination are free of charge. When you submit your visa application with the Australian Government's Department of Home Affairs, you will need to pay the visa fee.
+ [Changes to eligibility requirements]
+ All visa nomination eligibility requirements and priorities are subject to change throughout the year without notice.
+ Any changes made are effective immediately, regardless of when your SkillSelect Expression of Interest (EOI) was submitted (or amended). We strongly discourage changing your circumstances to meet the visa nomination criteria.
+ The Victorian Government endeavours to ensure all information on the Live in Melbourne website reflects the current eligibility requirements. The Live in Melbourne website is the authoritative source for information about Victoria's skilled visa nomination program.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="23" ht="409" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>state code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>state stream</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>requirements</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>service fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="409" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
       </c>
-      <c r="B23" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>WA_190</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr"/>
-      <c r="D23" s="1" t="inlineStr"/>
-      <c r="E23" s="1" t="inlineStr"/>
-      <c r="F23" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G23" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>OVERVIEW
 Under the SkillSelect model, the Department of Home Affairs invite skilled workers to apply for a Skilled Nominated visa (subclass 190) based on the claims presented in their expression of interest (EOI) in SkillSelect.
@@ -2923,41 +2991,39 @@
 You must be nominated to be invited to apply for this visa. Provided your nomination remains in effect, you may be eligible for the award of these points.</t>
         </is>
       </c>
-      <c r="H23" s="1" t="inlineStr"/>
-      <c r="I23" s="1" t="inlineStr"/>
-      <c r="J23" s="1" t="inlineStr"/>
-      <c r="K23" s="1" t="inlineStr"/>
-      <c r="L23" s="1" t="inlineStr"/>
-      <c r="M23" s="1" t="inlineStr"/>
-      <c r="N23" s="1" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
-    <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
+    <row r="3" ht="150" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
       </c>
-      <c r="B24" s="1" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>WA_491</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr"/>
-      <c r="D24" s="1" t="inlineStr"/>
-      <c r="E24" s="1" t="inlineStr"/>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>SKILLED WORK REGIONAL (PROVISIONAL) VISA - MAIN APPLICANT
+• ​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​stay in Australia for 5 years
+• live, work and study in a designated regional area of Australia
+• travel to and from Australia as many times as you want, while the visa is valid​
+• apply for permanent residence after 3 years from the time your visa is granted​.​
+SKILLED WORK REGIONAL (PROVISIONAL) VISA - SUBSEQUENT ENTRANT
+• ​be a member of the family unit of a person who holds a subclass 491 visa on the basis of satisfying the primary criteria for the grant of that visa.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G24" s="1" t="inlineStr"/>
-      <c r="H24" s="1" t="inlineStr"/>
-      <c r="I24" s="1" t="inlineStr"/>
-      <c r="J24" s="1" t="inlineStr"/>
-      <c r="K24" s="1" t="inlineStr"/>
-      <c r="L24" s="1" t="inlineStr"/>
-      <c r="M24" s="1" t="inlineStr"/>
-      <c r="N24" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>